<commit_message>
cards + client + tools: card text is authored in tokens (#81, #82)
`{keyword}` / `{keyword|display}` / `{V}{S}{M}` / `{card:ID}` replace the regex
keyword-bolding in RulesText. One dependency-free tokenizer
(packages/cards/src/text.ts, mirrored byte-for-byte into the client), loader
validation that collects every error across all cards, import-cards refusing bad
tokens, plainText() for every terminal consumer (MCP, sim heuristics, local
board). All 166 school/trainer texts converted by a mechanical pass whose plain
rendering equals the previous text exactly; the 34 ambiguous term matches are
listed in packages/cards/data/rewrites/2026-10-06-tokens.review.md for the user.
Pattern from the OpenSky review (OPENSKY_REVIEW.md C.14).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ibokki_spell_cards.xlsx
+++ b/ibokki_spell_cards.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1116" uniqueCount="1116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1276" uniqueCount="1276">
   <si>
     <t xml:space="preserve">Card ID</t>
   </si>
@@ -3372,6 +3372,486 @@
   </si>
   <si>
     <t xml:space="preserve">Heat saved from old blows, spent now on the body that took them.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deal 2 {damage|damage} to your opponent.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deal 3 {damage|damage} to your opponent. {discard} 1 random card.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deal 1 {damage|damage} to your opponent and give them 1 {burn}.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deal 1 {damage|damage} to your opponent. {disrupt|They discard} 1 random component.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This round, your damaging spells deal +1 {damage|damage}.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Return up to 2 Verbal-providing components {recover|from your discard pile} to your hand.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{discard} 1 card. Deal 1 {damage|damage} to your opponent for each symbol on it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{cost|Take 1 damage}. Deal 3 {damage|damage} to your opponent.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deal 2 {damage|damage} to your opponent. {draw} 1 card.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deal 1 {damage|damage} to your opponent and 2 {damage|damage} to a {ward} they control.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deal 5 {damage|damage} to your opponent.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deal 3 {damage|damage} to your opponent. {prevent|Reactions cannot target} this spell.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When your opponent casts a spell, deal 2 {damage|damage} to them. The spell still resolves.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{trap}: when your opponent {prevent|prevents} or reduces {damage|damage} you deal, deal 2 {damage|damage} to them.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{trap}: when your opponent attaches a Material (M) component to a prepared spell, deal 2 {damage|damage} to them.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When your opponent plays a Reaction, deal 4 {damage|damage} to them. The Reaction still resolves.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deal 6 {damage|damage} to your opponent.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deal 4 {damage|damage} to your opponent. This {damage|damage} {prevent|cannot be reduced} below 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deal 3 {damage|damage} to your opponent and give them 2 {burn}.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deal 2 {damage|damage} to your opponent. If they control a {ward}, 1 of that {damage|damage} hits the {ward} instead.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{discard} your hand. Deal 2 {damage|damage} to your opponent for each card {discard|discarded}.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Give your opponent 3 {burn}. This round, their {burn} also triggers at the start of your turns.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This round, your damaging spells deal +2 {damage|damage} and you {cost|take 1 damage} at the start of each of your turns.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deal 4 {damage|damage} to your opponent. {draw} 1 card.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deal 1 {damage|damage} to your opponent for each component attached to their prepared spells.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deal 3 {damage|damage} to your opponent. This round, their Reactions {lock|cost 1 additional} component to play.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deal 2 {damage|damage} to your opponent, plus 1 for each {burn} on them.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When your opponent casts a spell, deal {damage|damage} to them equal to its attached components. The spell still resolves.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{cancel} target spell that requires a Material (M) component. Deal 2 {damage|damage} to your opponent.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deal 3 {damage|damage} to your opponent. The spell still resolves.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When your opponent plays a Reaction, deal 3 {damage|damage} to them. The Reaction still resolves.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deal 7 {damage|damage} to your opponent.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deal 4 {damage|damage} to your opponent, then 2 {damage|damage} to each {ward} they control.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deal 5 {damage|damage} to your opponent. This spell {prevent|cannot be cancelled}, {cancel|redirected} or reduced.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Give your opponent 4 {burn}. This round, each of their {burn} deals 1 additional {damage|damage} when it triggers.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deal 3 {damage|damage} to your opponent, plus 2 for each Reaction they have cast this round.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deal 4 {damage|damage} to your opponent. {draw} 2 cards.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{cost|Take 3 damage}. Deal 8 {damage|damage} to your opponent.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Destroy all of your opponent's {ward|Wards}. Deal {damage|damage} to them equal to the HP those {ward|Wards} had.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This round, whenever your opponent plays a Reaction, deal 3 {damage|damage} to them.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When your opponent casts a spell, deal {damage|damage} to them equal to twice its level. The spell still resolves.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When target spell deals {damage|damage} to you, deal twice that {damage|damage} to your opponent.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When your opponent casts a spell or Reaction, deal 6 {damage|damage} to them. It still resolves.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deal 12 {damage|damage} to your opponent. This spell {prevent|cannot be cancelled}, {prevent|prevented}, {cancel|redirected} or reduced.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deal 6 {damage|damage} to your opponent. This round, your damaging spells deal +2 {damage|damage} and your {burn} {empower|deals double}.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When target spell deals {damage|damage} to you, deal three times that {damage|damage} to your opponent.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{draw} 2 cards.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{scry|Look at the top} 3 cards of your deck; take 1, put the rest back on top. This round, spell {damage|damage} dealt to you is {prevent|reduced by} 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{scry|Look at the top} 2 cards of your deck; take 1, put the other on the bottom. {heal|Remove 1 Burn} from yourself.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{prophecy} (2 turns): destroy your opponent's {unravel|largest Ward}.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{draw} 2 cards. If either is a multi-symbol component, {draw|draw} a third.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Return a component {recover|from your discard pile} to your hand.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deal 2 {damage|damage} to your opponent's {unravel|weakest Ward}. {scry|Look at the top} 2 cards of your deck and {scry|put them back} in any order.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{reveal|Look at the components in your opponent's hand}. {disrupt|They discard} one of your choice.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Your opponent's {unravel|largest Ward} {unravel|loses half its HP}, rounded up.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{draw} 1 card, then put a card from your hand on top of your deck.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deal 2 {damage|damage} to your opponent. {reveal|Look at their hand}.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{prophecy} (2 turns): deal 2 {damage|damage} to your opponent.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When your opponent casts a spell, {draw|draw} 1 card and deal 1 {damage|damage} to them. The spell still resolves.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Return up to 2 components {recover|from your discard pile} to your hand.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{scry|Search your deck} for a component and put it into your hand, then shuffle.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{reveal|Look at your opponent's hand}. {draw} 1 card.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{discard} any number of cards, then {draw|draw} that many.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Destroy target {ward} or ongoing effect. {draw} 1 card.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{prophecy} (2 turns): deal 4 {damage|damage} to your opponent.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{draw} 2 cards, then put a card from your hand on top of your deck.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{scry|Look at the top} 5 cards of your deck and {scry|put them back} in any order.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{scry|Look at the top} 3 cards of your deck and {scry|put them back} in any order. {prophecy} (1 turn): deal 2 {damage|damage} to your opponent.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Return a component attached to target spell {disrupt|to its owner's hand}. If the spell no longer meets its cost, {cancel|cancel} it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When your opponent casts a spell, {draw|draw} 1 card. The spell still resolves.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{cancel|Redirect} target spell: it hits its caster instead.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{recover|Cast a copy} of a Level 1 spell you have already cast this round, without paying its cost.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shuffle your {discard|discard} pile into your deck, then {draw|draw} 2 cards.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{scry|Search your deck} for any card and put it into your hand, then {draw|draw} 2 cards.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{scry|Look at the top} 5 cards of your deck; take 2, put the rest back on top in any order.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{reveal|Look at your opponent's hand} and the top 3 cards of their deck. {draw} 2 cards.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{prophecy} (3 turns): deal 7 {damage|damage} to your opponent.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{scry|Search your deck} for up to 2 components and put them into your hand, then shuffle.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{draw|Draw until} you have 7 cards in hand.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{cancel} target spell. It returns to its owner's prepared spells {seal|sealed}: it cannot be cast again this round.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{cancel} target spell and return its components {disrupt|to its owner's hand}. The spell returns to their prepared spells unspent.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{recover|Cast a copy} of a Level 1 or 2 spell either player has cast this round, without paying its cost.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{draw} 2 cards. Deal 1 {damage|damage} to your opponent for each card in your hand beyond 5.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{reveal|Look at your opponent's hand}. {disrupt|They discard} a card of your choice.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{draw} 4 cards. This turn, your spells {prevent|cannot be cancelled} or {cancel|redirected}.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Return every component {recover|from your discard pile} to your hand.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{scry|Search your deck} for up to 3 cards and put them into your hand, then shuffle.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{prophecy} (3 turns): deal 9 {damage|damage} to your opponent.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each player shuffles their hand and {discard|discard} pile into their deck, then {draw|draws} 5 cards.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{recover|Cast a copy} of any spell cast this round, without paying its cost. You may cast 1 {empower|additional spell} this turn.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{scry|Look at the top} 2 cards of your deck; take 1, put the other back on top.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{scry|Look at the top} card of your deck: a component goes to your hand, anything else to the bottom.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{discard} 1 card, then {draw|draw} 1 card.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Return a component {recover|from your discard pile} to the top of your deck.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The next damaging spell you cast this turn deals +1 {damage|damage}.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A {ward} you control gains 2 HP.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{discard} your hand, then {draw|draw} 4 cards.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{discard} 1 card, then {scry|search your deck} for any card and put it into your hand; shuffle.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{scry|Search your deck} for a same-symbol dual component (VV, SS or MM) and put it into your hand, then shuffle.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{scry|Look at the top} 4 cards of your deck and {scry|put them back} in any order.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{scry|Look at the top} card of your deck: a component attaches to one of your prepared spells, anything else goes to your hand.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{cost|Take 2 damage}. This turn you may cast 1 {empower|additional spell}, if you have a free slot and its components are attached.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{heal} 5.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{cost|Take 2 damage}. The next spell you cast this turn deals +3 {damage|damage}.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create a {ward} with 3 HP.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Destroy target {ward} or ongoing effect.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{heal|Remove all Burn} from yourself. {heal} 1 for each {burn} removed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Until the start of your next turn, your spells {prevent|cannot be cancelled} or {cancel|redirected}.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Until the start of your next turn, your opponent cannot make you {discard|discard} or {disrupt|strip} your cards or components.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shuffle your {discard|discard} pile into your deck.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Until the start of your next turn, your opponent {lock|cannot draw} cards beyond their normal turn {draw|draw}.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Until the start of your next turn, whenever your opponent plays a Reaction, they {cost|take 2 damage}.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{reveal|Look at your opponent's hand}. You may put a component from it {disrupt|on top of their deck}.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A {ward} you control gains 2 HP (create a 2 HP {ward} if you have none). {heal|Remove 1 Burn} from yourself.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create a {ward} with 1 HP. If it is destroyed this round, {draw|draw} 2 cards.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each {ward} you control gains 1 HP. If you control a {ward}, deal 1 {damage|damage} to your opponent.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Until the start of your next turn, spells with only 1 component attached {prevent|cannot target} you.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This round, spell {damage|damage} dealt to you is {prevent|reduced by} 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target spell deals 1 {prevent|less damage}.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target spell deals 1 {prevent|less damage}, or 2 less if you control a {ward}.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target spell deals 1 {prevent|less damage}. {draw} 1 card.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{trap}: when your opponent attaches a component to a prepared spell, return that component {disrupt|to their hand}.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{seal} target prepared spell your opponent controls: it cannot be cast this round.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{prevent} all {damage|damage} from target spell. {heal} half the {damage|damage} {prevent|prevented}, rounded down.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create a {ward} with 3 HP. Whenever it absorbs {damage|damage}, deal 1 {damage|damage} to your opponent.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove all components from target spell; if it no longer meets its cost, {cancel|cancel} it. {cost|Your opponent draws} 1 card.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{cancel} target spell. You may {empower|immediately attach} 1 component from your hand to a prepared spell.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{cancel} target spell that requires a Material (M) component.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{cancel} target spell that requires a Somatic (S) component.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Until the start of your next turn, your opponent {lock|cannot play Reactions}.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This round, your opponent's Reactions {lock|cost 1 additional} component to play.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create a {ward} with 2 HP. While it stands, Level 1 spells {prevent|cannot target} you.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create a {ward} with 3 HP. While it stands, the first time each round your opponent casts a spell, {draw|draw} 1 card.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{cost|Sacrifice} one of your {ward|Wards}. {prevent} all {damage|damage} from target spell.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create a {ward} with 6 HP. This round, {damage|damage} dealt to you is {prevent|reduced by} 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{cancel} target spell. Your opponent {lock|cannot cast} more spells this turn.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This round, spell {damage|damage} that would hit you {heal|heals} you instead (up to 5 HP).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each {ward} you control gains 2 HP.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{cancel} target spell. Deal 2 {damage|damage} to your opponent for each component attached to it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create a {ward} with 5 HP. When it is destroyed, create a {ward} with 2 HP.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{disrupt|Strip} every component from your opponent's prepared spells; {cancel|cancel} target spell if it no longer meets its cost. They {draw|draw} 1 card per spell stripped.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create a {ward} with 4 HP. This round, your opponent {prevent|cannot target} or destroy your {ward|Wards}.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Destroy one of your {ward|Wards}. Deal {damage|damage} equal to its remaining HP to your opponent.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deal {damage|damage} to your opponent equal to half your {ledger|ledger}, rounded up.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deal 3 {damage|damage} to your opponent for each Reaction you have played this round.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This round, whenever your opponent plays a Reaction, they {cost|take 3 damage}.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deal 5 {damage|damage} to your opponent, or 7 if you control a {ward}.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{cost|Sacrifice} all your {ward|Wards}. Deal 2 {damage|damage} to your opponent for each HP they had.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{cancel} target spell. Deal twice the {damage|damage} it would have dealt to your opponent.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deal 4 {damage|damage} to your opponent. If they control a {ward}, destroy it and deal 8 {damage|damage} instead.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This round, spells {prevent|cannot damage you} and your opponent {lock|cannot play Reactions}.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create a {ward} with 10 HP that your opponent {prevent|cannot target} or destroy. When it breaks, {heal|heal} 5.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{cancel} every spell on the stack. Your opponent {lock|cannot cast} spells this turn or play Reactions until the start of your next turn.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deal {damage|damage} to your opponent equal to your current HP.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deal 4 {damage|damage} to your opponent for each round of this match so far.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{cancel} every spell your opponent has on the stack. Deal 3 {damage|damage} to them for each spell {cancel|cancelled}.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Destroy every {ward} on both sides. Deal 3 {damage|damage} to your opponent for each {ward} destroyed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spend up to 4 from your {ledger|ledger}. Create a {ward} with HP equal to the amount spent.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spend 6 from your {ledger|ledger} to {cancel|cancel} target spell. Castable only with 6 or more banked.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spend up to 6 from your {ledger|ledger}. {heal} half the amount spent, rounded down.</t>
   </si>
 </sst>
 </file>
@@ -3847,7 +4327,7 @@
         <v>13</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>828</v>
+        <v>1229</v>
       </c>
       <c r="H2" s="6"/>
       <c r="I2" s="5" t="s">
@@ -3880,7 +4360,7 @@
         <v>13</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>829</v>
+        <v>1230</v>
       </c>
       <c r="H3" s="6"/>
       <c r="I3" s="5" t="s">
@@ -3913,7 +4393,7 @@
         <v>13</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>830</v>
+        <v>1231</v>
       </c>
       <c r="H4" s="6"/>
       <c r="I4" s="5" t="s">
@@ -3946,7 +4426,7 @@
         <v>13</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>831</v>
+        <v>1232</v>
       </c>
       <c r="H5" s="6"/>
       <c r="I5" s="5" t="s">
@@ -3979,7 +4459,7 @@
         <v>13</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>832</v>
+        <v>1233</v>
       </c>
       <c r="H6" s="6"/>
       <c r="I6" s="5" t="s">
@@ -4012,7 +4492,7 @@
         <v>13</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>833</v>
+        <v>1234</v>
       </c>
       <c r="H7" s="6"/>
       <c r="I7" s="5" t="s">
@@ -4045,7 +4525,7 @@
         <v>13</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>834</v>
+        <v>1235</v>
       </c>
       <c r="H8" s="6"/>
       <c r="I8" s="5" t="s">
@@ -4078,7 +4558,7 @@
         <v>13</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>835</v>
+        <v>1236</v>
       </c>
       <c r="H9" s="6"/>
       <c r="I9" s="5" t="s">
@@ -4111,7 +4591,7 @@
         <v>13</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>836</v>
+        <v>1237</v>
       </c>
       <c r="H10" s="6"/>
       <c r="I10" s="5" t="s">
@@ -4144,7 +4624,7 @@
         <v>51</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>837</v>
+        <v>1238</v>
       </c>
       <c r="H11" s="6"/>
       <c r="I11" s="5" t="s">
@@ -4177,7 +4657,7 @@
         <v>51</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>838</v>
+        <v>1239</v>
       </c>
       <c r="H12" s="6"/>
       <c r="I12" s="5" t="s">
@@ -4210,7 +4690,7 @@
         <v>51</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>839</v>
+        <v>1240</v>
       </c>
       <c r="H13" s="6"/>
       <c r="I13" s="5" t="s">
@@ -4243,7 +4723,7 @@
         <v>51</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>840</v>
+        <v>1241</v>
       </c>
       <c r="H14" s="6"/>
       <c r="I14" s="5" t="s">
@@ -4276,7 +4756,7 @@
         <v>51</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>841</v>
+        <v>1242</v>
       </c>
       <c r="H15" s="6"/>
       <c r="I15" s="5" t="s">
@@ -4309,7 +4789,7 @@
         <v>72</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>842</v>
+        <v>1243</v>
       </c>
       <c r="H16" s="6"/>
       <c r="I16" s="5" t="s">
@@ -4342,7 +4822,7 @@
         <v>51</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>843</v>
+        <v>1244</v>
       </c>
       <c r="H17" s="6"/>
       <c r="I17" s="5" t="s">
@@ -4375,7 +4855,7 @@
         <v>51</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>844</v>
+        <v>1245</v>
       </c>
       <c r="H18" s="6"/>
       <c r="I18" s="5" t="s">
@@ -4408,7 +4888,7 @@
         <v>51</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>845</v>
+        <v>1246</v>
       </c>
       <c r="H19" s="6"/>
       <c r="I19" s="5" t="s">
@@ -4441,7 +4921,7 @@
         <v>51</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>846</v>
+        <v>1247</v>
       </c>
       <c r="H20" s="6"/>
       <c r="I20" s="5" t="s">
@@ -4474,7 +4954,7 @@
         <v>93</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>847</v>
+        <v>1248</v>
       </c>
       <c r="H21" s="6"/>
       <c r="I21" s="5" t="s">
@@ -4507,7 +4987,7 @@
         <v>51</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>848</v>
+        <v>1249</v>
       </c>
       <c r="H22" s="6"/>
       <c r="I22" s="5" t="s">
@@ -4540,7 +5020,7 @@
         <v>102</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>849</v>
+        <v>1250</v>
       </c>
       <c r="H23" s="6"/>
       <c r="I23" s="5" t="s">
@@ -4573,7 +5053,7 @@
         <v>102</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>850</v>
+        <v>1251</v>
       </c>
       <c r="H24" s="6"/>
       <c r="I24" s="5" t="s">
@@ -4606,7 +5086,7 @@
         <v>111</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>851</v>
+        <v>1252</v>
       </c>
       <c r="H25" s="6"/>
       <c r="I25" s="5" t="s">
@@ -4639,7 +5119,7 @@
         <v>102</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>852</v>
+        <v>1253</v>
       </c>
       <c r="H26" s="6"/>
       <c r="I26" s="5" t="s">
@@ -4672,7 +5152,7 @@
         <v>120</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>853</v>
+        <v>1254</v>
       </c>
       <c r="H27" s="6"/>
       <c r="I27" s="5" t="s">
@@ -4705,7 +5185,7 @@
         <v>111</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>854</v>
+        <v>1255</v>
       </c>
       <c r="H28" s="6"/>
       <c r="I28" s="5" t="s">
@@ -4738,7 +5218,7 @@
         <v>102</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>855</v>
+        <v>1256</v>
       </c>
       <c r="H29" s="6"/>
       <c r="I29" s="5" t="s">
@@ -4771,7 +5251,7 @@
         <v>102</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>856</v>
+        <v>1257</v>
       </c>
       <c r="H30" s="6"/>
       <c r="I30" s="5" t="s">
@@ -4804,7 +5284,7 @@
         <v>111</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>837</v>
+        <v>1238</v>
       </c>
       <c r="H31" s="6"/>
       <c r="I31" s="5" t="s">
@@ -4837,7 +5317,7 @@
         <v>102</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>857</v>
+        <v>1258</v>
       </c>
       <c r="H32" s="6"/>
       <c r="I32" s="5" t="s">
@@ -4870,7 +5350,7 @@
         <v>51</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>858</v>
+        <v>1259</v>
       </c>
       <c r="H33" s="6"/>
       <c r="I33" s="5" t="s">
@@ -4903,7 +5383,7 @@
         <v>111</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>859</v>
+        <v>1260</v>
       </c>
       <c r="H34" s="6"/>
       <c r="I34" s="5" t="s">
@@ -4936,7 +5416,7 @@
         <v>102</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>860</v>
+        <v>1261</v>
       </c>
       <c r="H35" s="6"/>
       <c r="I35" s="5" t="s">
@@ -4969,7 +5449,7 @@
         <v>102</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>861</v>
+        <v>1262</v>
       </c>
       <c r="H36" s="6"/>
       <c r="I36" s="5" t="s">
@@ -5002,7 +5482,7 @@
         <v>120</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>862</v>
+        <v>1263</v>
       </c>
       <c r="H37" s="6"/>
       <c r="I37" s="5" t="s">
@@ -5035,7 +5515,7 @@
         <v>102</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>863</v>
+        <v>1264</v>
       </c>
       <c r="H38" s="6"/>
       <c r="I38" s="5" t="s">
@@ -5068,7 +5548,7 @@
         <v>111</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>864</v>
+        <v>1265</v>
       </c>
       <c r="H39" s="6"/>
       <c r="I39" s="5" t="s">
@@ -5101,7 +5581,7 @@
         <v>173</v>
       </c>
       <c r="G40" s="5" t="s">
-        <v>865</v>
+        <v>1266</v>
       </c>
       <c r="H40" s="6"/>
       <c r="I40" s="5" t="s">
@@ -5134,7 +5614,7 @@
         <v>178</v>
       </c>
       <c r="G41" s="5" t="s">
-        <v>866</v>
+        <v>1267</v>
       </c>
       <c r="H41" s="6"/>
       <c r="I41" s="5" t="s">
@@ -5167,7 +5647,7 @@
         <v>173</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>867</v>
+        <v>1268</v>
       </c>
       <c r="H42" s="6"/>
       <c r="I42" s="5" t="s">
@@ -5200,7 +5680,7 @@
         <v>173</v>
       </c>
       <c r="G43" s="5" t="s">
-        <v>868</v>
+        <v>1269</v>
       </c>
       <c r="H43" s="6"/>
       <c r="I43" s="5" t="s">
@@ -5233,7 +5713,7 @@
         <v>178</v>
       </c>
       <c r="G44" s="5" t="s">
-        <v>869</v>
+        <v>1270</v>
       </c>
       <c r="H44" s="6"/>
       <c r="I44" s="5" t="s">
@@ -5266,7 +5746,7 @@
         <v>173</v>
       </c>
       <c r="G45" s="5" t="s">
-        <v>870</v>
+        <v>1271</v>
       </c>
       <c r="H45" s="6"/>
       <c r="I45" s="5" t="s">
@@ -5299,7 +5779,7 @@
         <v>173</v>
       </c>
       <c r="G46" s="5" t="s">
-        <v>871</v>
+        <v>1272</v>
       </c>
       <c r="H46" s="6"/>
       <c r="I46" s="5" t="s">
@@ -5340,7 +5820,7 @@
         </is>
       </c>
       <c r="G47" s="5" t="s">
-        <v>872</v>
+        <v>1273</v>
       </c>
       <c r="H47" s="6"/>
       <c r="I47" s="5" t="inlineStr">
@@ -5383,7 +5863,7 @@
         </is>
       </c>
       <c r="G48" s="5" t="s">
-        <v>873</v>
+        <v>1274</v>
       </c>
       <c r="H48" s="6"/>
       <c r="I48" s="5" t="inlineStr">
@@ -5426,7 +5906,7 @@
         </is>
       </c>
       <c r="G49" s="5" t="s">
-        <v>874</v>
+        <v>1275</v>
       </c>
       <c r="H49" s="6"/>
       <c r="I49" s="5" t="inlineStr">
@@ -5526,7 +6006,7 @@
         <v>204</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>714</v>
+        <v>1116</v>
       </c>
       <c r="H2" s="6"/>
       <c r="I2" s="5" t="s">
@@ -5559,7 +6039,7 @@
         <v>204</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>715</v>
+        <v>1117</v>
       </c>
       <c r="H3" s="6"/>
       <c r="I3" s="5" t="s">
@@ -5592,7 +6072,7 @@
         <v>204</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>716</v>
+        <v>1118</v>
       </c>
       <c r="H4" s="6"/>
       <c r="I4" s="5" t="s">
@@ -5625,7 +6105,7 @@
         <v>204</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>717</v>
+        <v>1119</v>
       </c>
       <c r="H5" s="6"/>
       <c r="I5" s="5"/>
@@ -5656,7 +6136,7 @@
         <v>204</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>718</v>
+        <v>1120</v>
       </c>
       <c r="H6" s="6"/>
       <c r="I6" s="5"/>
@@ -5687,7 +6167,7 @@
         <v>204</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>719</v>
+        <v>1121</v>
       </c>
       <c r="H7" s="6"/>
       <c r="I7" s="5"/>
@@ -5718,7 +6198,7 @@
         <v>204</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>720</v>
+        <v>1122</v>
       </c>
       <c r="H8" s="6"/>
       <c r="I8" s="5" t="s">
@@ -5751,7 +6231,7 @@
         <v>204</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>721</v>
+        <v>1123</v>
       </c>
       <c r="H9" s="6"/>
       <c r="I9" s="5"/>
@@ -5782,7 +6262,7 @@
         <v>233</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>722</v>
+        <v>1124</v>
       </c>
       <c r="H10" s="6"/>
       <c r="I10" s="5" t="s">
@@ -5815,7 +6295,7 @@
         <v>204</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>723</v>
+        <v>1125</v>
       </c>
       <c r="H11" s="6"/>
       <c r="I11" s="5"/>
@@ -5846,7 +6326,7 @@
         <v>241</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>724</v>
+        <v>1126</v>
       </c>
       <c r="H12" s="6"/>
       <c r="I12" s="5"/>
@@ -5877,7 +6357,7 @@
         <v>241</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>725</v>
+        <v>1127</v>
       </c>
       <c r="H13" s="6"/>
       <c r="I13" s="5" t="s">
@@ -5910,7 +6390,7 @@
         <v>204</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>726</v>
+        <v>1128</v>
       </c>
       <c r="H14" s="6"/>
       <c r="I14" s="5"/>
@@ -5941,7 +6421,7 @@
         <v>204</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>727</v>
+        <v>1129</v>
       </c>
       <c r="H15" s="6"/>
       <c r="I15" s="5" t="s">
@@ -5974,7 +6454,7 @@
         <v>204</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>728</v>
+        <v>1130</v>
       </c>
       <c r="H16" s="6"/>
       <c r="I16" s="5" t="s">
@@ -6007,7 +6487,7 @@
         <v>241</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>729</v>
+        <v>1131</v>
       </c>
       <c r="H17" s="6"/>
       <c r="I17" s="5"/>
@@ -6038,7 +6518,7 @@
         <v>241</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>730</v>
+        <v>1132</v>
       </c>
       <c r="H18" s="6"/>
       <c r="I18" s="5" t="s">
@@ -6071,7 +6551,7 @@
         <v>241</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>731</v>
+        <v>1133</v>
       </c>
       <c r="H19" s="6"/>
       <c r="I19" s="5" t="s">
@@ -6104,7 +6584,7 @@
         <v>241</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>732</v>
+        <v>1134</v>
       </c>
       <c r="H20" s="6"/>
       <c r="I20" s="5"/>
@@ -6135,7 +6615,7 @@
         <v>241</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>733</v>
+        <v>1135</v>
       </c>
       <c r="H21" s="6"/>
       <c r="I21" s="5" t="s">
@@ -6168,7 +6648,7 @@
         <v>241</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>734</v>
+        <v>1136</v>
       </c>
       <c r="H22" s="6"/>
       <c r="I22" s="5" t="s">
@@ -6201,7 +6681,7 @@
         <v>241</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>735</v>
+        <v>1137</v>
       </c>
       <c r="H23" s="6"/>
       <c r="I23" s="5" t="s">
@@ -6234,7 +6714,7 @@
         <v>241</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>736</v>
+        <v>1138</v>
       </c>
       <c r="H24" s="6"/>
       <c r="I24" s="5" t="s">
@@ -6267,7 +6747,7 @@
         <v>233</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>737</v>
+        <v>1139</v>
       </c>
       <c r="H25" s="6"/>
       <c r="I25" s="5" t="s">
@@ -6300,7 +6780,7 @@
         <v>241</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>738</v>
+        <v>1140</v>
       </c>
       <c r="H26" s="6"/>
       <c r="I26" s="5" t="s">
@@ -6333,7 +6813,7 @@
         <v>93</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>739</v>
+        <v>1141</v>
       </c>
       <c r="H27" s="6"/>
       <c r="I27" s="5" t="s">
@@ -6366,7 +6846,7 @@
         <v>241</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>740</v>
+        <v>1142</v>
       </c>
       <c r="H28" s="6"/>
       <c r="I28" s="5" t="s">
@@ -6399,7 +6879,7 @@
         <v>241</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>741</v>
+        <v>1143</v>
       </c>
       <c r="H29" s="6"/>
       <c r="I29" s="5" t="s">
@@ -6432,7 +6912,7 @@
         <v>233</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>742</v>
+        <v>1144</v>
       </c>
       <c r="H30" s="6"/>
       <c r="I30" s="5" t="s">
@@ -6465,7 +6945,7 @@
         <v>241</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>743</v>
+        <v>1145</v>
       </c>
       <c r="H31" s="6"/>
       <c r="I31" s="5"/>
@@ -6496,7 +6976,7 @@
         <v>241</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>744</v>
+        <v>1146</v>
       </c>
       <c r="H32" s="6"/>
       <c r="I32" s="5" t="s">
@@ -6529,7 +7009,7 @@
         <v>321</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>745</v>
+        <v>1147</v>
       </c>
       <c r="H33" s="6"/>
       <c r="I33" s="5" t="s">
@@ -6562,7 +7042,7 @@
         <v>321</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>746</v>
+        <v>1148</v>
       </c>
       <c r="H34" s="6"/>
       <c r="I34" s="5" t="s">
@@ -6595,7 +7075,7 @@
         <v>321</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>734</v>
+        <v>1136</v>
       </c>
       <c r="H35" s="6"/>
       <c r="I35" s="5" t="s">
@@ -6628,7 +7108,7 @@
         <v>321</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>747</v>
+        <v>1149</v>
       </c>
       <c r="H36" s="6"/>
       <c r="I36" s="5" t="s">
@@ -6661,7 +7141,7 @@
         <v>321</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>748</v>
+        <v>1150</v>
       </c>
       <c r="H37" s="6"/>
       <c r="I37" s="5" t="s">
@@ -6694,7 +7174,7 @@
         <v>321</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>749</v>
+        <v>1151</v>
       </c>
       <c r="H38" s="6"/>
       <c r="I38" s="5" t="s">
@@ -6727,7 +7207,7 @@
         <v>346</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>750</v>
+        <v>1152</v>
       </c>
       <c r="H39" s="6"/>
       <c r="I39" s="5" t="s">
@@ -6760,7 +7240,7 @@
         <v>321</v>
       </c>
       <c r="G40" s="5" t="s">
-        <v>751</v>
+        <v>1153</v>
       </c>
       <c r="H40" s="6"/>
       <c r="I40" s="5" t="s">
@@ -6793,7 +7273,7 @@
         <v>321</v>
       </c>
       <c r="G41" s="5" t="s">
-        <v>752</v>
+        <v>1154</v>
       </c>
       <c r="H41" s="6"/>
       <c r="I41" s="5" t="s">
@@ -6826,7 +7306,7 @@
         <v>359</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>753</v>
+        <v>1155</v>
       </c>
       <c r="H42" s="6"/>
       <c r="I42" s="5" t="s">
@@ -6859,7 +7339,7 @@
         <v>321</v>
       </c>
       <c r="G43" s="5" t="s">
-        <v>754</v>
+        <v>1156</v>
       </c>
       <c r="H43" s="6"/>
       <c r="I43" s="5" t="s">
@@ -6892,7 +7372,7 @@
         <v>346</v>
       </c>
       <c r="G44" s="5" t="s">
-        <v>755</v>
+        <v>1157</v>
       </c>
       <c r="H44" s="6"/>
       <c r="I44" s="5"/>
@@ -6923,7 +7403,7 @@
         <v>321</v>
       </c>
       <c r="G45" s="5" t="s">
-        <v>756</v>
+        <v>1158</v>
       </c>
       <c r="H45" s="6"/>
       <c r="I45" s="5"/>
@@ -6954,7 +7434,7 @@
         <v>374</v>
       </c>
       <c r="G46" s="5" t="s">
-        <v>757</v>
+        <v>1159</v>
       </c>
       <c r="H46" s="6"/>
       <c r="I46" s="5" t="s">
@@ -6987,7 +7467,7 @@
         <v>379</v>
       </c>
       <c r="G47" s="5" t="s">
-        <v>758</v>
+        <v>1160</v>
       </c>
       <c r="H47" s="6"/>
       <c r="I47" s="5" t="s">
@@ -7020,7 +7500,7 @@
         <v>384</v>
       </c>
       <c r="G48" s="5" t="s">
-        <v>759</v>
+        <v>1161</v>
       </c>
       <c r="H48" s="6"/>
       <c r="I48" s="5" t="s">
@@ -7118,7 +7598,7 @@
         <v>390</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>760</v>
+        <v>1162</v>
       </c>
       <c r="H2" s="6"/>
       <c r="I2" s="5" t="s">
@@ -7151,7 +7631,7 @@
         <v>390</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>761</v>
+        <v>1163</v>
       </c>
       <c r="H3" s="6"/>
       <c r="I3" s="5" t="s">
@@ -7184,7 +7664,7 @@
         <v>390</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>762</v>
+        <v>1164</v>
       </c>
       <c r="H4" s="6"/>
       <c r="I4" s="5" t="s">
@@ -7217,7 +7697,7 @@
         <v>390</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>763</v>
+        <v>1165</v>
       </c>
       <c r="H5" s="6"/>
       <c r="I5" s="5" t="s">
@@ -7250,7 +7730,7 @@
         <v>390</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>764</v>
+        <v>1166</v>
       </c>
       <c r="H6" s="6"/>
       <c r="I6" s="5" t="s">
@@ -7283,7 +7763,7 @@
         <v>390</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>765</v>
+        <v>1167</v>
       </c>
       <c r="H7" s="6"/>
       <c r="I7" s="5" t="s">
@@ -7316,7 +7796,7 @@
         <v>390</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>766</v>
+        <v>1168</v>
       </c>
       <c r="H8" s="6"/>
       <c r="I8" s="5" t="s">
@@ -7349,7 +7829,7 @@
         <v>390</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>767</v>
+        <v>1169</v>
       </c>
       <c r="H9" s="6"/>
       <c r="I9" s="5" t="s">
@@ -7382,7 +7862,7 @@
         <v>390</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>768</v>
+        <v>1170</v>
       </c>
       <c r="H10" s="6"/>
       <c r="I10" s="5" t="s">
@@ -7415,7 +7895,7 @@
         <v>390</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>769</v>
+        <v>1171</v>
       </c>
       <c r="H11" s="6"/>
       <c r="I11" s="5" t="s">
@@ -7448,7 +7928,7 @@
         <v>390</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>770</v>
+        <v>1172</v>
       </c>
       <c r="H12" s="6"/>
       <c r="I12" s="5" t="s">
@@ -7481,7 +7961,7 @@
         <v>447</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>771</v>
+        <v>1173</v>
       </c>
       <c r="H13" s="6"/>
       <c r="I13" s="5" t="s">
@@ -7541,7 +8021,7 @@
         <v>390</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>772</v>
+        <v>1174</v>
       </c>
       <c r="H15" s="6"/>
       <c r="I15" s="5" t="s">
@@ -7574,7 +8054,7 @@
         <v>447</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>773</v>
+        <v>1175</v>
       </c>
       <c r="H16" s="6"/>
       <c r="I16" s="5" t="s">
@@ -7607,7 +8087,7 @@
         <v>447</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>774</v>
+        <v>1176</v>
       </c>
       <c r="H17" s="6"/>
       <c r="I17" s="5" t="s">
@@ -7640,7 +8120,7 @@
         <v>447</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>775</v>
+        <v>1177</v>
       </c>
       <c r="H18" s="6"/>
       <c r="I18" s="5" t="s">
@@ -7673,7 +8153,7 @@
         <v>447</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>776</v>
+        <v>1178</v>
       </c>
       <c r="H19" s="6"/>
       <c r="I19" s="5" t="s">
@@ -7706,7 +8186,7 @@
         <v>447</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>777</v>
+        <v>1179</v>
       </c>
       <c r="H20" s="6"/>
       <c r="I20" s="5" t="s">
@@ -7739,7 +8219,7 @@
         <v>447</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>778</v>
+        <v>1180</v>
       </c>
       <c r="H21" s="6"/>
       <c r="I21" s="5" t="s">
@@ -7772,7 +8252,7 @@
         <v>447</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>779</v>
+        <v>1181</v>
       </c>
       <c r="H22" s="6"/>
       <c r="I22" s="5" t="s">
@@ -7805,7 +8285,7 @@
         <v>447</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>780</v>
+        <v>1182</v>
       </c>
       <c r="H23" s="6"/>
       <c r="I23" s="5" t="s">
@@ -7838,7 +8318,7 @@
         <v>447</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>781</v>
+        <v>1183</v>
       </c>
       <c r="H24" s="6"/>
       <c r="I24" s="5" t="s">
@@ -7871,7 +8351,7 @@
         <v>447</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>782</v>
+        <v>1184</v>
       </c>
       <c r="H25" s="6"/>
       <c r="I25" s="5" t="s">
@@ -7904,7 +8384,7 @@
         <v>447</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>783</v>
+        <v>1185</v>
       </c>
       <c r="H26" s="6"/>
       <c r="I26" s="5" t="s">
@@ -7937,7 +8417,7 @@
         <v>492</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>784</v>
+        <v>1186</v>
       </c>
       <c r="H27" s="6"/>
       <c r="I27" s="5" t="s">
@@ -7970,7 +8450,7 @@
         <v>497</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>785</v>
+        <v>1187</v>
       </c>
       <c r="H28" s="6"/>
       <c r="I28" s="5" t="s">
@@ -8003,7 +8483,7 @@
         <v>502</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>786</v>
+        <v>1188</v>
       </c>
       <c r="H29" s="6"/>
       <c r="I29" s="5" t="s">
@@ -8036,7 +8516,7 @@
         <v>502</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>787</v>
+        <v>1189</v>
       </c>
       <c r="H30" s="6"/>
       <c r="I30" s="5" t="s">
@@ -8069,7 +8549,7 @@
         <v>502</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>788</v>
+        <v>1190</v>
       </c>
       <c r="H31" s="6"/>
       <c r="I31" s="5" t="s">
@@ -8102,7 +8582,7 @@
         <v>502</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>789</v>
+        <v>1191</v>
       </c>
       <c r="H32" s="6"/>
       <c r="I32" s="5" t="s">
@@ -8135,7 +8615,7 @@
         <v>502</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>790</v>
+        <v>1192</v>
       </c>
       <c r="H33" s="6"/>
       <c r="I33" s="5" t="s">
@@ -8168,7 +8648,7 @@
         <v>502</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>791</v>
+        <v>1193</v>
       </c>
       <c r="H34" s="6"/>
       <c r="I34" s="5" t="s">
@@ -8201,7 +8681,7 @@
         <v>502</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>792</v>
+        <v>1194</v>
       </c>
       <c r="H35" s="6"/>
       <c r="I35" s="5" t="s">
@@ -8234,7 +8714,7 @@
         <v>502</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>793</v>
+        <v>1195</v>
       </c>
       <c r="H36" s="6"/>
       <c r="I36" s="5" t="s">
@@ -8267,7 +8747,7 @@
         <v>502</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>794</v>
+        <v>1196</v>
       </c>
       <c r="H37" s="6"/>
       <c r="I37" s="5" t="s">
@@ -8300,7 +8780,7 @@
         <v>539</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>795</v>
+        <v>1197</v>
       </c>
       <c r="H38" s="6"/>
       <c r="I38" s="5" t="s">
@@ -8333,7 +8813,7 @@
         <v>539</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>796</v>
+        <v>1198</v>
       </c>
       <c r="H39" s="6"/>
       <c r="I39" s="5" t="s">
@@ -8366,7 +8846,7 @@
         <v>548</v>
       </c>
       <c r="G40" s="5" t="s">
-        <v>797</v>
+        <v>1199</v>
       </c>
       <c r="H40" s="6"/>
       <c r="I40" s="5" t="s">
@@ -8399,7 +8879,7 @@
         <v>553</v>
       </c>
       <c r="G41" s="5" t="s">
-        <v>798</v>
+        <v>1200</v>
       </c>
       <c r="H41" s="6"/>
       <c r="I41" s="5" t="s">
@@ -8432,7 +8912,7 @@
         <v>553</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>799</v>
+        <v>1201</v>
       </c>
       <c r="H42" s="6"/>
       <c r="I42" s="5" t="s">
@@ -8465,7 +8945,7 @@
         <v>553</v>
       </c>
       <c r="G43" s="5" t="s">
-        <v>800</v>
+        <v>1202</v>
       </c>
       <c r="H43" s="6"/>
       <c r="I43" s="5" t="s">
@@ -8498,7 +8978,7 @@
         <v>553</v>
       </c>
       <c r="G44" s="5" t="s">
-        <v>801</v>
+        <v>1203</v>
       </c>
       <c r="H44" s="6"/>
       <c r="I44" s="5" t="s">
@@ -8531,7 +9011,7 @@
         <v>553</v>
       </c>
       <c r="G45" s="5" t="s">
-        <v>802</v>
+        <v>1204</v>
       </c>
       <c r="H45" s="6"/>
       <c r="I45" s="5" t="s">
@@ -8564,7 +9044,7 @@
         <v>574</v>
       </c>
       <c r="G46" s="5" t="s">
-        <v>803</v>
+        <v>1205</v>
       </c>
       <c r="H46" s="6"/>
       <c r="I46" s="5" t="s">
@@ -8652,7 +9132,7 @@
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
       <c r="G2" s="5" t="s">
-        <v>804</v>
+        <v>1206</v>
       </c>
       <c r="H2" s="6" t="s">
         <v>582</v>
@@ -8677,7 +9157,7 @@
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
       <c r="G3" s="5" t="s">
-        <v>805</v>
+        <v>1207</v>
       </c>
       <c r="H3" s="6" t="s">
         <v>587</v>
@@ -8702,7 +9182,7 @@
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
       <c r="G4" s="5" t="s">
-        <v>769</v>
+        <v>1171</v>
       </c>
       <c r="H4" s="6" t="s">
         <v>587</v>
@@ -8727,7 +9207,7 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
       <c r="G5" s="5" t="s">
-        <v>806</v>
+        <v>1208</v>
       </c>
       <c r="H5" s="6" t="s">
         <v>596</v>
@@ -8777,7 +9257,7 @@
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
       <c r="G7" s="5" t="s">
-        <v>808</v>
+        <v>1209</v>
       </c>
       <c r="H7" s="6" t="s">
         <v>606</v>
@@ -8802,7 +9282,7 @@
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
       <c r="G8" s="5" t="s">
-        <v>809</v>
+        <v>1210</v>
       </c>
       <c r="H8" s="6" t="s">
         <v>611</v>
@@ -8827,7 +9307,7 @@
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
       <c r="G9" s="5" t="s">
-        <v>810</v>
+        <v>1211</v>
       </c>
       <c r="H9" s="6" t="s">
         <v>616</v>
@@ -8911,7 +9391,7 @@
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
       <c r="G2" s="5" t="s">
-        <v>779</v>
+        <v>1181</v>
       </c>
       <c r="H2" s="6" t="s">
         <v>622</v>
@@ -8936,7 +9416,7 @@
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
       <c r="G3" s="5" t="s">
-        <v>811</v>
+        <v>1212</v>
       </c>
       <c r="H3" s="6" t="s">
         <v>627</v>
@@ -8961,7 +9441,7 @@
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
       <c r="G4" s="5" t="s">
-        <v>812</v>
+        <v>1213</v>
       </c>
       <c r="H4" s="6" t="s">
         <v>582</v>
@@ -8986,7 +9466,7 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
       <c r="G5" s="5" t="s">
-        <v>813</v>
+        <v>1214</v>
       </c>
       <c r="H5" s="6" t="s">
         <v>636</v>
@@ -9011,7 +9491,7 @@
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
       <c r="G6" s="5" t="s">
-        <v>765</v>
+        <v>1167</v>
       </c>
       <c r="H6" s="6" t="s">
         <v>606</v>
@@ -9036,7 +9516,7 @@
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
       <c r="G7" s="5" t="s">
-        <v>814</v>
+        <v>1215</v>
       </c>
       <c r="H7" s="6" t="s">
         <v>644</v>
@@ -9061,7 +9541,7 @@
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
       <c r="G8" s="5" t="s">
-        <v>815</v>
+        <v>1216</v>
       </c>
       <c r="H8" s="6" t="s">
         <v>649</v>
@@ -9086,7 +9566,7 @@
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
       <c r="G9" s="5" t="s">
-        <v>816</v>
+        <v>1217</v>
       </c>
       <c r="H9" s="6" t="s">
         <v>654</v>
@@ -9111,7 +9591,7 @@
       <c r="E10" s="4"/>
       <c r="F10" s="4"/>
       <c r="G10" s="5" t="s">
-        <v>817</v>
+        <v>1218</v>
       </c>
       <c r="H10" s="6" t="s">
         <v>659</v>
@@ -9136,7 +9616,7 @@
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
       <c r="G11" s="5" t="s">
-        <v>818</v>
+        <v>1219</v>
       </c>
       <c r="H11" s="6" t="s">
         <v>611</v>
@@ -9161,7 +9641,7 @@
       <c r="E12" s="4"/>
       <c r="F12" s="4"/>
       <c r="G12" s="5" t="s">
-        <v>819</v>
+        <v>1220</v>
       </c>
       <c r="H12" s="6" t="s">
         <v>668</v>
@@ -9186,7 +9666,7 @@
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
       <c r="G13" s="5" t="s">
-        <v>820</v>
+        <v>1221</v>
       </c>
       <c r="H13" s="6" t="s">
         <v>673</v>
@@ -9211,7 +9691,7 @@
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
       <c r="G14" s="5" t="s">
-        <v>821</v>
+        <v>1222</v>
       </c>
       <c r="H14" s="6" t="s">
         <v>678</v>
@@ -9236,7 +9716,7 @@
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
       <c r="G15" s="5" t="s">
-        <v>822</v>
+        <v>1223</v>
       </c>
       <c r="H15" s="6" t="s">
         <v>683</v>
@@ -9261,7 +9741,7 @@
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
       <c r="G16" s="5" t="s">
-        <v>823</v>
+        <v>1224</v>
       </c>
       <c r="H16" s="6" t="s">
         <v>688</v>
@@ -9286,7 +9766,7 @@
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
       <c r="G17" s="5" t="s">
-        <v>824</v>
+        <v>1225</v>
       </c>
       <c r="H17" s="6" t="s">
         <v>693</v>
@@ -9311,7 +9791,7 @@
       <c r="E18" s="4"/>
       <c r="F18" s="4"/>
       <c r="G18" s="5" t="s">
-        <v>825</v>
+        <v>1226</v>
       </c>
       <c r="H18" s="6" t="s">
         <v>698</v>
@@ -9336,7 +9816,7 @@
       <c r="E19" s="4"/>
       <c r="F19" s="4"/>
       <c r="G19" s="5" t="s">
-        <v>826</v>
+        <v>1227</v>
       </c>
       <c r="H19" s="6" t="s">
         <v>683</v>
@@ -9361,7 +9841,7 @@
       <c r="E20" s="4"/>
       <c r="F20" s="4"/>
       <c r="G20" s="5" t="s">
-        <v>771</v>
+        <v>1173</v>
       </c>
       <c r="H20" s="6" t="s">
         <v>707</v>
@@ -9386,7 +9866,7 @@
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
       <c r="G21" s="5" t="s">
-        <v>827</v>
+        <v>1228</v>
       </c>
       <c r="H21" s="6" t="s">
         <v>712</v>

</xml_diff>

<commit_message>
cards: token review pass — 17 texts (user-approved 2026-10-07)
From packages/cards/data/rewrites/2026-10-06-tokens.review.md: Scalding Air and
Spite deal Damage to the opponent (was Cost); "damage" inside prevention
sentences, opponent-subject draw/discard and "discard pile" are plain prose
again; Channel Pyromancy's +2 is Empower. Costs you pay, redirect-as-Cancel and
Sunburst's Ward icon stay as converted. Engine untouched; ledger re-stamped.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ibokki_spell_cards.xlsx
+++ b/ibokki_spell_cards.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1276" uniqueCount="1276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1292" uniqueCount="1292">
   <si>
     <t xml:space="preserve">Card ID</t>
   </si>
@@ -3852,6 +3852,54 @@
   </si>
   <si>
     <t xml:space="preserve">Spend up to 6 from your {ledger|ledger}. {heal} half the amount spent, rounded down.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{trap}: when your opponent {prevent|prevents} or reduces damage you deal, deal 2 {damage|damage} to them.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deal 4 {damage|damage} to your opponent. This damage {prevent|cannot be reduced} below 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This round, your damaging spells deal {empower|+2 damage} and you {cost|take 1 damage} at the start of each of your turns.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{discard} your hand. Deal 2 {damage|damage} to your opponent for each card discarded.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{scry|Look at the top} 3 cards of your deck; take 1, put the rest back on top. This round, spell damage dealt to you is {prevent|reduced by} 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each player shuffles their hand and discard pile into their deck, then {draw|draws} 5 cards.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Until the start of your next turn, whenever your opponent plays a Reaction, they take 2 {damage|damage}.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Until the start of your next turn, your opponent {lock|cannot draw} cards beyond their normal turn draw.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Until the start of your next turn, your opponent cannot make you discard or {disrupt|strip} your cards or components.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This round, whenever your opponent plays a Reaction, they take 3 {damage|damage}.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This round, spell damage dealt to you is {prevent|reduced by} 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create a {ward} with 6 HP. This round, damage dealt to you is {prevent|reduced by} 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{prevent} all damage from target spell. {heal} half the damage {prevent|prevented}, rounded down.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{cost|Sacrifice} one of your {ward|Wards}. {prevent} all damage from target spell.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create a {ward} with 3 HP. Whenever it absorbs damage, deal 1 {damage|damage} to your opponent.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{disrupt|Strip} every component from your opponent's prepared spells; {cancel|cancel} target spell if it no longer meets its cost. They draw 1 card per spell stripped.</t>
   </si>
 </sst>
 </file>
@@ -4459,7 +4507,7 @@
         <v>13</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>1233</v>
+        <v>1286</v>
       </c>
       <c r="H6" s="6"/>
       <c r="I6" s="5" t="s">
@@ -4657,7 +4705,7 @@
         <v>51</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>1239</v>
+        <v>1288</v>
       </c>
       <c r="H12" s="6"/>
       <c r="I12" s="5" t="s">
@@ -4690,7 +4738,7 @@
         <v>51</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>1240</v>
+        <v>1290</v>
       </c>
       <c r="H13" s="6"/>
       <c r="I13" s="5" t="s">
@@ -4987,7 +5035,7 @@
         <v>51</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>1249</v>
+        <v>1289</v>
       </c>
       <c r="H22" s="6"/>
       <c r="I22" s="5" t="s">
@@ -5020,7 +5068,7 @@
         <v>102</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>1250</v>
+        <v>1287</v>
       </c>
       <c r="H23" s="6"/>
       <c r="I23" s="5" t="s">
@@ -5218,7 +5266,7 @@
         <v>102</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>1256</v>
+        <v>1291</v>
       </c>
       <c r="H29" s="6"/>
       <c r="I29" s="5" t="s">
@@ -5416,7 +5464,7 @@
         <v>102</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>1261</v>
+        <v>1285</v>
       </c>
       <c r="H35" s="6"/>
       <c r="I35" s="5" t="s">
@@ -6421,7 +6469,7 @@
         <v>204</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>1129</v>
+        <v>1276</v>
       </c>
       <c r="H15" s="6"/>
       <c r="I15" s="5" t="s">
@@ -6551,7 +6599,7 @@
         <v>241</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>1133</v>
+        <v>1277</v>
       </c>
       <c r="H19" s="6"/>
       <c r="I19" s="5" t="s">
@@ -6648,7 +6696,7 @@
         <v>241</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>1136</v>
+        <v>1279</v>
       </c>
       <c r="H22" s="6"/>
       <c r="I22" s="5" t="s">
@@ -6714,7 +6762,7 @@
         <v>241</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>1138</v>
+        <v>1278</v>
       </c>
       <c r="H24" s="6"/>
       <c r="I24" s="5" t="s">
@@ -7075,7 +7123,7 @@
         <v>321</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>1136</v>
+        <v>1279</v>
       </c>
       <c r="H35" s="6"/>
       <c r="I35" s="5" t="s">
@@ -7631,7 +7679,7 @@
         <v>390</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>1163</v>
+        <v>1280</v>
       </c>
       <c r="H3" s="6"/>
       <c r="I3" s="5" t="s">
@@ -9011,7 +9059,7 @@
         <v>553</v>
       </c>
       <c r="G45" s="5" t="s">
-        <v>1204</v>
+        <v>1281</v>
       </c>
       <c r="H45" s="6"/>
       <c r="I45" s="5" t="s">
@@ -9741,7 +9789,7 @@
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
       <c r="G16" s="5" t="s">
-        <v>1224</v>
+        <v>1284</v>
       </c>
       <c r="H16" s="6" t="s">
         <v>688</v>
@@ -9791,7 +9839,7 @@
       <c r="E18" s="4"/>
       <c r="F18" s="4"/>
       <c r="G18" s="5" t="s">
-        <v>1226</v>
+        <v>1283</v>
       </c>
       <c r="H18" s="6" t="s">
         <v>698</v>
@@ -9816,7 +9864,7 @@
       <c r="E19" s="4"/>
       <c r="F19" s="4"/>
       <c r="G19" s="5" t="s">
-        <v>1227</v>
+        <v>1282</v>
       </c>
       <c r="H19" s="6" t="s">
         <v>683</v>

</xml_diff>

<commit_message>
cards + client + protocol: drop flavor text from every card (DECISIONS #8)
The flavor lines added with the Fire reorientation (DECISIONS #6) are removed
rather than hidden, per the user after seeing them live: 139 sheet cells
cleared by a retext pass, the importer no longer reads the column, CardDef /
catalog / client lose the field, and the spellbook tray, detail rail and deck
builder preview render none.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ibokki_spell_cards.xlsx
+++ b/ibokki_spell_cards.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1292" uniqueCount="1292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1293" uniqueCount="1293">
   <si>
     <t xml:space="preserve">Card ID</t>
   </si>
@@ -3900,6 +3900,9 @@
   </si>
   <si>
     <t xml:space="preserve">{disrupt|Strip} every component from your opponent's prepared spells; {cancel|cancel} target spell if it no longer meets its cost. They draw 1 card per spell stripped.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"/>
   </si>
 </sst>
 </file>
@@ -4385,7 +4388,7 @@
         <v>884</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>1068</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4418,7 +4421,7 @@
         <v>884</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>1069</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4451,7 +4454,7 @@
         <v>884</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>1070</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4484,7 +4487,7 @@
         <v>884</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>1071</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4517,7 +4520,7 @@
         <v>884</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>1072</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4550,7 +4553,7 @@
         <v>884</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>1073</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4583,7 +4586,7 @@
         <v>884</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>1074</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4616,7 +4619,7 @@
         <v>884</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>1075</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4649,7 +4652,7 @@
         <v>884</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>1076</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4682,7 +4685,7 @@
         <v>884</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>1077</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4715,7 +4718,7 @@
         <v>884</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>1078</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4748,7 +4751,7 @@
         <v>884</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>1079</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4781,7 +4784,7 @@
         <v>884</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>1080</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4814,7 +4817,7 @@
         <v>884</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>1081</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4847,7 +4850,7 @@
         <v>884</v>
       </c>
       <c r="K16" s="5" t="s">
-        <v>1082</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4880,7 +4883,7 @@
         <v>884</v>
       </c>
       <c r="K17" s="5" t="s">
-        <v>1083</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4913,7 +4916,7 @@
         <v>884</v>
       </c>
       <c r="K18" s="5" t="s">
-        <v>1084</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4946,7 +4949,7 @@
         <v>884</v>
       </c>
       <c r="K19" s="5" t="s">
-        <v>1085</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4979,7 +4982,7 @@
         <v>884</v>
       </c>
       <c r="K20" s="5" t="s">
-        <v>1086</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5012,7 +5015,7 @@
         <v>884</v>
       </c>
       <c r="K21" s="5" t="s">
-        <v>1087</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5045,7 +5048,7 @@
         <v>884</v>
       </c>
       <c r="K22" s="5" t="s">
-        <v>1088</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5078,7 +5081,7 @@
         <v>884</v>
       </c>
       <c r="K23" s="5" t="s">
-        <v>1089</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5111,7 +5114,7 @@
         <v>884</v>
       </c>
       <c r="K24" s="5" t="s">
-        <v>1090</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5144,7 +5147,7 @@
         <v>884</v>
       </c>
       <c r="K25" s="5" t="s">
-        <v>1091</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5177,7 +5180,7 @@
         <v>884</v>
       </c>
       <c r="K26" s="5" t="s">
-        <v>1092</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5210,7 +5213,7 @@
         <v>884</v>
       </c>
       <c r="K27" s="5" t="s">
-        <v>1093</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5243,7 +5246,7 @@
         <v>884</v>
       </c>
       <c r="K28" s="5" t="s">
-        <v>1094</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5276,7 +5279,7 @@
         <v>884</v>
       </c>
       <c r="K29" s="5" t="s">
-        <v>1095</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5309,7 +5312,7 @@
         <v>884</v>
       </c>
       <c r="K30" s="5" t="s">
-        <v>1096</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5342,7 +5345,7 @@
         <v>884</v>
       </c>
       <c r="K31" s="5" t="s">
-        <v>1097</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5375,7 +5378,7 @@
         <v>884</v>
       </c>
       <c r="K32" s="5" t="s">
-        <v>1098</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5408,7 +5411,7 @@
         <v>884</v>
       </c>
       <c r="K33" s="5" t="s">
-        <v>1099</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5441,7 +5444,7 @@
         <v>884</v>
       </c>
       <c r="K34" s="5" t="s">
-        <v>1100</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5474,7 +5477,7 @@
         <v>884</v>
       </c>
       <c r="K35" s="5" t="s">
-        <v>1101</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5507,7 +5510,7 @@
         <v>884</v>
       </c>
       <c r="K36" s="5" t="s">
-        <v>1102</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5540,7 +5543,7 @@
         <v>884</v>
       </c>
       <c r="K37" s="5" t="s">
-        <v>1103</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5573,7 +5576,7 @@
         <v>884</v>
       </c>
       <c r="K38" s="5" t="s">
-        <v>1104</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5606,7 +5609,7 @@
         <v>884</v>
       </c>
       <c r="K39" s="5" t="s">
-        <v>1105</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5639,7 +5642,7 @@
         <v>884</v>
       </c>
       <c r="K40" s="5" t="s">
-        <v>1106</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5672,7 +5675,7 @@
         <v>884</v>
       </c>
       <c r="K41" s="5" t="s">
-        <v>1107</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5705,7 +5708,7 @@
         <v>884</v>
       </c>
       <c r="K42" s="5" t="s">
-        <v>1108</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5738,7 +5741,7 @@
         <v>884</v>
       </c>
       <c r="K43" s="5" t="s">
-        <v>1109</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5771,7 +5774,7 @@
         <v>884</v>
       </c>
       <c r="K44" s="5" t="s">
-        <v>1110</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5804,7 +5807,7 @@
         <v>884</v>
       </c>
       <c r="K45" s="5" t="s">
-        <v>1111</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5837,7 +5840,7 @@
         <v>884</v>
       </c>
       <c r="K46" s="5" t="s">
-        <v>1112</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5880,7 +5883,7 @@
         <v>884</v>
       </c>
       <c r="K47" s="5" t="s">
-        <v>1113</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5923,7 +5926,7 @@
         <v>884</v>
       </c>
       <c r="K48" s="5" t="s">
-        <v>1114</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5966,7 +5969,7 @@
         <v>884</v>
       </c>
       <c r="K49" s="5" t="s">
-        <v>1115</v>
+        <v>1292</v>
       </c>
     </row>
   </sheetData>
@@ -6064,7 +6067,7 @@
         <v>884</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>886</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6097,7 +6100,7 @@
         <v>884</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>887</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6130,7 +6133,7 @@
         <v>884</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>888</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6161,7 +6164,7 @@
         <v>884</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>889</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6192,7 +6195,7 @@
         <v>884</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>890</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6223,7 +6226,7 @@
         <v>884</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>891</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6256,7 +6259,7 @@
         <v>884</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>892</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6287,7 +6290,7 @@
         <v>884</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>893</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6320,7 +6323,7 @@
         <v>884</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>894</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6351,7 +6354,7 @@
         <v>884</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>895</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6382,7 +6385,7 @@
         <v>884</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>896</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6415,7 +6418,7 @@
         <v>884</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>897</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6446,7 +6449,7 @@
         <v>884</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>898</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6479,7 +6482,7 @@
         <v>884</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>899</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6512,7 +6515,7 @@
         <v>884</v>
       </c>
       <c r="K16" s="5" t="s">
-        <v>900</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6543,7 +6546,7 @@
         <v>884</v>
       </c>
       <c r="K17" s="5" t="s">
-        <v>901</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6576,7 +6579,7 @@
         <v>884</v>
       </c>
       <c r="K18" s="5" t="s">
-        <v>902</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6609,7 +6612,7 @@
         <v>884</v>
       </c>
       <c r="K19" s="5" t="s">
-        <v>903</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6640,7 +6643,7 @@
         <v>884</v>
       </c>
       <c r="K20" s="5" t="s">
-        <v>904</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6673,7 +6676,7 @@
         <v>884</v>
       </c>
       <c r="K21" s="5" t="s">
-        <v>905</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6706,7 +6709,7 @@
         <v>884</v>
       </c>
       <c r="K22" s="5" t="s">
-        <v>906</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6739,7 +6742,7 @@
         <v>884</v>
       </c>
       <c r="K23" s="5" t="s">
-        <v>907</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6772,7 +6775,7 @@
         <v>884</v>
       </c>
       <c r="K24" s="5" t="s">
-        <v>908</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6805,7 +6808,7 @@
         <v>884</v>
       </c>
       <c r="K25" s="5" t="s">
-        <v>909</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6838,7 +6841,7 @@
         <v>884</v>
       </c>
       <c r="K26" s="5" t="s">
-        <v>910</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6871,7 +6874,7 @@
         <v>884</v>
       </c>
       <c r="K27" s="5" t="s">
-        <v>911</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6904,7 +6907,7 @@
         <v>884</v>
       </c>
       <c r="K28" s="5" t="s">
-        <v>912</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6937,7 +6940,7 @@
         <v>884</v>
       </c>
       <c r="K29" s="5" t="s">
-        <v>913</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6970,7 +6973,7 @@
         <v>884</v>
       </c>
       <c r="K30" s="5" t="s">
-        <v>914</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7001,7 +7004,7 @@
         <v>884</v>
       </c>
       <c r="K31" s="5" t="s">
-        <v>915</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7034,7 +7037,7 @@
         <v>884</v>
       </c>
       <c r="K32" s="5" t="s">
-        <v>916</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7067,7 +7070,7 @@
         <v>884</v>
       </c>
       <c r="K33" s="5" t="s">
-        <v>917</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7100,7 +7103,7 @@
         <v>884</v>
       </c>
       <c r="K34" s="5" t="s">
-        <v>918</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7133,7 +7136,7 @@
         <v>884</v>
       </c>
       <c r="K35" s="5" t="s">
-        <v>919</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7166,7 +7169,7 @@
         <v>884</v>
       </c>
       <c r="K36" s="5" t="s">
-        <v>920</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7199,7 +7202,7 @@
         <v>884</v>
       </c>
       <c r="K37" s="5" t="s">
-        <v>921</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7232,7 +7235,7 @@
         <v>884</v>
       </c>
       <c r="K38" s="5" t="s">
-        <v>922</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7265,7 +7268,7 @@
         <v>884</v>
       </c>
       <c r="K39" s="5" t="s">
-        <v>923</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7298,7 +7301,7 @@
         <v>884</v>
       </c>
       <c r="K40" s="5" t="s">
-        <v>924</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7331,7 +7334,7 @@
         <v>884</v>
       </c>
       <c r="K41" s="5" t="s">
-        <v>925</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7364,7 +7367,7 @@
         <v>884</v>
       </c>
       <c r="K42" s="5" t="s">
-        <v>926</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7397,7 +7400,7 @@
         <v>884</v>
       </c>
       <c r="K43" s="5" t="s">
-        <v>927</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7428,7 +7431,7 @@
         <v>884</v>
       </c>
       <c r="K44" s="5" t="s">
-        <v>928</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7459,7 +7462,7 @@
         <v>884</v>
       </c>
       <c r="K45" s="5" t="s">
-        <v>929</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7492,7 +7495,7 @@
         <v>884</v>
       </c>
       <c r="K46" s="5" t="s">
-        <v>930</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7525,7 +7528,7 @@
         <v>884</v>
       </c>
       <c r="K47" s="5" t="s">
-        <v>931</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7558,7 +7561,7 @@
         <v>884</v>
       </c>
       <c r="K48" s="5" t="s">
-        <v>932</v>
+        <v>1292</v>
       </c>
     </row>
   </sheetData>
@@ -7656,7 +7659,7 @@
         <v>884</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>977</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7689,7 +7692,7 @@
         <v>884</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>978</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7722,7 +7725,7 @@
         <v>884</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>979</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7755,7 +7758,7 @@
         <v>884</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>980</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7788,7 +7791,7 @@
         <v>884</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>981</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7821,7 +7824,7 @@
         <v>884</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>982</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7854,7 +7857,7 @@
         <v>884</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>983</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7887,7 +7890,7 @@
         <v>884</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>984</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7920,7 +7923,7 @@
         <v>884</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>985</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7953,7 +7956,7 @@
         <v>884</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>986</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7986,7 +7989,7 @@
         <v>884</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>987</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8019,7 +8022,7 @@
         <v>884</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>988</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8079,7 +8082,7 @@
         <v>884</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>989</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8112,7 +8115,7 @@
         <v>884</v>
       </c>
       <c r="K16" s="5" t="s">
-        <v>990</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8145,7 +8148,7 @@
         <v>884</v>
       </c>
       <c r="K17" s="5" t="s">
-        <v>991</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8178,7 +8181,7 @@
         <v>884</v>
       </c>
       <c r="K18" s="5" t="s">
-        <v>992</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8211,7 +8214,7 @@
         <v>884</v>
       </c>
       <c r="K19" s="5" t="s">
-        <v>993</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8244,7 +8247,7 @@
         <v>884</v>
       </c>
       <c r="K20" s="5" t="s">
-        <v>994</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8277,7 +8280,7 @@
         <v>884</v>
       </c>
       <c r="K21" s="5" t="s">
-        <v>995</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8310,7 +8313,7 @@
         <v>884</v>
       </c>
       <c r="K22" s="5" t="s">
-        <v>996</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8343,7 +8346,7 @@
         <v>884</v>
       </c>
       <c r="K23" s="5" t="s">
-        <v>997</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8376,7 +8379,7 @@
         <v>884</v>
       </c>
       <c r="K24" s="5" t="s">
-        <v>998</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8409,7 +8412,7 @@
         <v>884</v>
       </c>
       <c r="K25" s="5" t="s">
-        <v>999</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8442,7 +8445,7 @@
         <v>884</v>
       </c>
       <c r="K26" s="5" t="s">
-        <v>1000</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8475,7 +8478,7 @@
         <v>884</v>
       </c>
       <c r="K27" s="5" t="s">
-        <v>1001</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8508,7 +8511,7 @@
         <v>884</v>
       </c>
       <c r="K28" s="5" t="s">
-        <v>1002</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8541,7 +8544,7 @@
         <v>884</v>
       </c>
       <c r="K29" s="5" t="s">
-        <v>1003</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8574,7 +8577,7 @@
         <v>884</v>
       </c>
       <c r="K30" s="5" t="s">
-        <v>1004</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8607,7 +8610,7 @@
         <v>884</v>
       </c>
       <c r="K31" s="5" t="s">
-        <v>1005</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8640,7 +8643,7 @@
         <v>884</v>
       </c>
       <c r="K32" s="5" t="s">
-        <v>1006</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8673,7 +8676,7 @@
         <v>884</v>
       </c>
       <c r="K33" s="5" t="s">
-        <v>1007</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8706,7 +8709,7 @@
         <v>884</v>
       </c>
       <c r="K34" s="5" t="s">
-        <v>1008</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8739,7 +8742,7 @@
         <v>884</v>
       </c>
       <c r="K35" s="5" t="s">
-        <v>1009</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8772,7 +8775,7 @@
         <v>884</v>
       </c>
       <c r="K36" s="5" t="s">
-        <v>1010</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8805,7 +8808,7 @@
         <v>884</v>
       </c>
       <c r="K37" s="5" t="s">
-        <v>1011</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8838,7 +8841,7 @@
         <v>884</v>
       </c>
       <c r="K38" s="5" t="s">
-        <v>1012</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8871,7 +8874,7 @@
         <v>884</v>
       </c>
       <c r="K39" s="5" t="s">
-        <v>1013</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8904,7 +8907,7 @@
         <v>884</v>
       </c>
       <c r="K40" s="5" t="s">
-        <v>1014</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8937,7 +8940,7 @@
         <v>884</v>
       </c>
       <c r="K41" s="5" t="s">
-        <v>1015</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8970,7 +8973,7 @@
         <v>884</v>
       </c>
       <c r="K42" s="5" t="s">
-        <v>1016</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9003,7 +9006,7 @@
         <v>884</v>
       </c>
       <c r="K43" s="5" t="s">
-        <v>1017</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9036,7 +9039,7 @@
         <v>884</v>
       </c>
       <c r="K44" s="5" t="s">
-        <v>1018</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9069,7 +9072,7 @@
         <v>884</v>
       </c>
       <c r="K45" s="5" t="s">
-        <v>1019</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9102,7 +9105,7 @@
         <v>884</v>
       </c>
       <c r="K46" s="5" t="s">
-        <v>1020</v>
+        <v>1292</v>
       </c>
     </row>
   </sheetData>

</xml_diff>